<commit_message>
feat: Effective Date from FY+Quarter, per-supplier Form# persistence, simplified dropdown (v1.0.5)
</commit_message>
<xml_diff>
--- a/data/supplier info/Contract Source info.xlsx
+++ b/data/supplier info/Contract Source info.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -747,17 +747,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="2df2684a-2237-489e-8795-1f946593e18f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3ddbdfa1-be50-4b7a-b66f-14c4748c8596">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C7BB62D9C7AC4249BB50D4F119F8FF50" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dab14850594d04436880d3464ba468af">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ddbdfa1-be50-4b7a-b66f-14c4748c8596" xmlns:ns3="2df2684a-2237-489e-8795-1f946593e18f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb8d2f689c1774a9065a5e99593f72e7" ns2:_="" ns3:_="">
     <xsd:import namespace="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
@@ -986,6 +975,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="2df2684a-2237-489e-8795-1f946593e18f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3ddbdfa1-be50-4b7a-b66f-14c4748c8596">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6A94BBB-A0AD-4FB8-BDF4-92E3AE460DEC}">
   <ds:schemaRefs>
@@ -995,17 +995,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2853F184-2900-4A13-8F7C-F055FF8A0E87}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2df2684a-2237-489e-8795-1f946593e18f"/>
-    <ds:schemaRef ds:uri="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF7C219A-DDF7-4D1E-BD82-ACDB83DC22F4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1022,4 +1011,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2853F184-2900-4A13-8F7C-F055FF8A0E87}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2df2684a-2237-489e-8795-1f946593e18f"/>
+    <ds:schemaRef ds:uri="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
chore: update supplier info + Word template (v1.0.6)
</commit_message>
<xml_diff>
--- a/data/supplier info/Contract Source info.xlsx
+++ b/data/supplier info/Contract Source info.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hp.sharepoint.com/teams/InputDevice/Shared Documents/General/17. Automation Projects/rebate-form-generator/data/supplier info/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hp.sharepoint.com/teams/InputDevice/Shared Documents/General/17. Automation Projects/Mason WorkingFile/RebateFormGenerator_v1.0.5/RebateFormGenerator/data/supplier info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{FC584247-0D60-4284-AB83-01F87EC44D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D74F746C-9278-43DE-B0E2-15DF8E6DB725}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{FC584247-0D60-4284-AB83-01F87EC44D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB13CB2A-B100-422E-9428-D6731CB866BC}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{22D0AACF-9824-475A-8BD7-108A3230197E}"/>
   </bookViews>
@@ -122,12 +122,6 @@
     <t>Chicony</t>
   </si>
   <si>
-    <t>Jensen Tsai</t>
-  </si>
-  <si>
-    <t>Mobile Keyboard BU G.M.</t>
-  </si>
-  <si>
     <t>Liteon</t>
   </si>
   <si>
@@ -165,6 +159,12 @@
   </si>
   <si>
     <t>Chairman &amp; CEO</t>
+  </si>
+  <si>
+    <t>Lawrence Wang</t>
+  </si>
+  <si>
+    <t>Sales AVP, MKB BU</t>
   </si>
 </sst>
 </file>
@@ -585,7 +585,7 @@
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
@@ -680,56 +680,56 @@
         <v>25</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
         <v>30</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>31</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s">
         <v>32</v>
       </c>
-      <c r="D6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" t="s">
-        <v>32</v>
-      </c>
-      <c r="F6" t="s">
-        <v>34</v>
-      </c>
       <c r="G6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" t="s">
         <v>40</v>
-      </c>
-      <c r="C7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" t="s">
-        <v>35</v>
-      </c>
-      <c r="F7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G7" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -738,15 +738,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C7BB62D9C7AC4249BB50D4F119F8FF50" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dab14850594d04436880d3464ba468af">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ddbdfa1-be50-4b7a-b66f-14c4748c8596" xmlns:ns3="2df2684a-2237-489e-8795-1f946593e18f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb8d2f689c1774a9065a5e99593f72e7" ns2:_="" ns3:_="">
     <xsd:import namespace="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
@@ -975,6 +966,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -987,14 +987,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6A94BBB-A0AD-4FB8-BDF4-92E3AE460DEC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF7C219A-DDF7-4D1E-BD82-ACDB83DC22F4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1013,6 +1005,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6A94BBB-A0AD-4FB8-BDF4-92E3AE460DEC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2853F184-2900-4A13-8F7C-F055FF8A0E87}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat: new iCertis template support - new keywords, SDT replacement, iCertis Code field (v1.1.0)
</commit_message>
<xml_diff>
--- a/data/supplier info/Contract Source info.xlsx
+++ b/data/supplier info/Contract Source info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hp.sharepoint.com/teams/InputDevice/Shared Documents/General/17. Automation Projects/Mason WorkingFile/RebateFormGenerator_v1.0.5/RebateFormGenerator/data/supplier info/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hp.sharepoint.com/teams/InputDevice/Shared Documents/General/17. Automation Projects/rebate-form-generator/data/supplier info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{FC584247-0D60-4284-AB83-01F87EC44D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB13CB2A-B100-422E-9428-D6731CB866BC}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="8_{FC584247-0D60-4284-AB83-01F87EC44D58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E97A3D67-8F60-4A46-9776-8D932AE433BE}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{22D0AACF-9824-475A-8BD7-108A3230197E}"/>
+    <workbookView xWindow="4800" yWindow="3110" windowWidth="14400" windowHeight="8170" xr2:uid="{22D0AACF-9824-475A-8BD7-108A3230197E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,41 +36,20 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
-  <si>
-    <t>Address</t>
-  </si>
-  <si>
-    <t>Signer</t>
-  </si>
-  <si>
-    <t>Title</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Supplier Name</t>
   </si>
   <si>
-    <t>Name of Entity</t>
-  </si>
-  <si>
     <t>Acrox</t>
   </si>
   <si>
-    <t>4F., No.89, Minshan St., Neihu Dist., Taipei City 114, Taiwan, R.O.C.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acrox Technologies Co., Limited </t>
-  </si>
-  <si>
     <t>Sarita Liu</t>
   </si>
   <si>
     <t>Chairman</t>
   </si>
   <si>
-    <t>Contract Number</t>
-  </si>
-  <si>
     <t>CW2295436</t>
   </si>
   <si>
@@ -80,12 +59,6 @@
     <t>CW2295430</t>
   </si>
   <si>
-    <t>DARFON ELECTRONICS CORP.</t>
-  </si>
-  <si>
-    <t>No.167, Shanying Rd.,Guishan Dist, Taoyuan City 333, Taiwan, R.O.C.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Chris Wang </t>
   </si>
   <si>
@@ -98,12 +71,6 @@
     <t>CW2247631</t>
   </si>
   <si>
-    <t>SUNREX TECHNOLOGY CORP.</t>
-  </si>
-  <si>
-    <t>No.475, Sec. 4, Changping Rd., Daya Dist., Taichung City 428</t>
-  </si>
-  <si>
     <t>Ellie Chen</t>
   </si>
   <si>
@@ -113,12 +80,6 @@
     <t>CW2295509</t>
   </si>
   <si>
-    <t>Chicony Electronics Co., Ltd.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">37F, No.69, Sec. 2, Guangfu Rd., Sanchong Dist., New Taipei City 24158 </t>
-  </si>
-  <si>
     <t>Chicony</t>
   </si>
   <si>
@@ -128,30 +89,9 @@
     <t>CW2295409</t>
   </si>
   <si>
-    <t>LITE-ON TECHNOLOGY CORPORATION</t>
-  </si>
-  <si>
-    <t>22FL., 392, RUEY KUANG RD., NEIHU DIST., TAIPEI 114</t>
-  </si>
-  <si>
-    <t>Jerry Hsu</t>
-  </si>
-  <si>
-    <t>PRIMAX ELECTRONICS LTD.</t>
-  </si>
-  <si>
-    <t>669, Ruey Kuang Road, Neihu 114, Taipei, Taiwan, R.O.C.</t>
-  </si>
-  <si>
     <t>Primax</t>
   </si>
   <si>
-    <t>SUPPLIER-Sign</t>
-  </si>
-  <si>
-    <t>Senior Vice President/ IT&amp;CE SBG Head</t>
-  </si>
-  <si>
     <t>CW2286756</t>
   </si>
   <si>
@@ -165,6 +105,63 @@
   </si>
   <si>
     <t>Sales AVP, MKB BU</t>
+  </si>
+  <si>
+    <t>CW#</t>
+  </si>
+  <si>
+    <t>LITEON TECHNOLOGY CORPORATION</t>
+  </si>
+  <si>
+    <t>PRIMAX ELECTRONICS LTD</t>
+  </si>
+  <si>
+    <t>CHICONY ELECTRONICS CO LTD</t>
+  </si>
+  <si>
+    <t>SUNREX TECHNOLOGY CORP</t>
+  </si>
+  <si>
+    <t>DARFON ELECTRONICS CORP</t>
+  </si>
+  <si>
+    <t>ACROX TECHNOLOGIES CO LTD</t>
+  </si>
+  <si>
+    <t>ICMPartyName1</t>
+  </si>
+  <si>
+    <t>ICMExternalSignatory</t>
+  </si>
+  <si>
+    <t>ICMExternalSignatoryTitle</t>
+  </si>
+  <si>
+    <t>ICMRebateAgreementCode</t>
+  </si>
+  <si>
+    <t>Rebate_000042</t>
+  </si>
+  <si>
+    <t>Rebate_000106</t>
+  </si>
+  <si>
+    <t>Rebate_000046</t>
+  </si>
+  <si>
+    <t>Rebate_000029</t>
+  </si>
+  <si>
+    <t>Rebate_000080</t>
+  </si>
+  <si>
+    <t>Rebate_000044</t>
+  </si>
+  <si>
+    <t>Anson Chiu</t>
+  </si>
+  <si>
+    <t>President</t>
   </si>
 </sst>
 </file>
@@ -559,177 +556,155 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85372B2B-50B0-4229-A423-1626AABDF9FE}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="32.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.1796875" customWidth="1"/>
-    <col min="5" max="5" width="32.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>2</v>
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
         <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E5" t="s">
-        <v>25</v>
+      <c r="E5" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="F5" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" t="s">
         <v>41</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>42</v>
-      </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" t="s">
-        <v>32</v>
-      </c>
-      <c r="G6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
         <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="F7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G7" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>